<commit_message>
Replace Kakao login with username/password signup in design docs
Signup registers parcels and creates the first field; requests are
identified by an X-User-Id header (hackathon demo, minimal security).
Update architecture, flow spec, team plan, outline, PRD feedback, and
both backlogs accordingly.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/dev/farmguardian_backlog_BE.xlsx
+++ b/docs/dev/farmguardian_backlog_BE.xlsx
@@ -81,7 +81,7 @@
     <t>BE-02</t>
   </si>
   <si>
-    <t>카카오 개발자 앱 등록</t>
+    <t>카카오 개발자 앱 등록 (불필요: 카카오 로그인 제거, 행 삭제 필요)</t>
   </si>
   <si>
     <t>BE-03</t>
@@ -180,7 +180,7 @@
     <t>BE-15</t>
   </si>
   <si>
-    <t>JWT 인증·소유자 검사 구현</t>
+    <t>X-User-Id 인증·소유자 검사 구현</t>
   </si>
   <si>
     <t>BE-16</t>
@@ -195,7 +195,7 @@
     <t>인증</t>
   </si>
   <si>
-    <t>카카오 SSO 로그인 구현</t>
+    <t>가입·로그인 구현 (가입 때 첫 밭 생성)</t>
   </si>
   <si>
     <t>BE-18</t>
@@ -207,7 +207,7 @@
     <t>BE-19</t>
   </si>
   <si>
-    <t>회원 탈퇴 구현 (카카오 연결 끊기)</t>
+    <t>회원 탈퇴 구현</t>
   </si>
   <si>
     <t>BE-20</t>

</xml_diff>

<commit_message>
Replace PSIS/NCPMS API ingest with Excel-based data load
Load drug and pest data from the team's seven Excel sheets via JSON
instead of calling PSIS and NCPMS. Drop the PSIS/NCPMS keys, parser
and sample-research tasks, add the sheet-to-table mapping and load
checks, and update the API spec, plan, outline, flow spec and backlog.
The Excel files themselves are not committed.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/dev/farmguardian_backlog_BE.xlsx
+++ b/docs/dev/farmguardian_backlog_BE.xlsx
@@ -66,7 +66,7 @@
     <t>준비</t>
   </si>
   <si>
-    <t>외부 API 키 신청 (도로명주소·팜맵·기상청·PSIS·NCPMS)</t>
+    <t>외부 API 키 신청 (도로명주소·팜맵·기상청)</t>
   </si>
   <si>
     <t>P0</t>
@@ -117,7 +117,7 @@
     <t>조사</t>
   </si>
   <si>
-    <t>PSIS 샘플 데이터 조사</t>
+    <t>엑셀 데이터 검수 (등록약·사용규칙, 확인 필요 행)</t>
   </si>
   <si>
     <t>혜빈님</t>
@@ -126,7 +126,7 @@
     <t>BE-08</t>
   </si>
   <si>
-    <t>NCPMS 샘플 데이터 조사</t>
+    <t>엑셀 데이터 검수 (도감·발생시기·매개충)</t>
   </si>
   <si>
     <t>BE-09</t>
@@ -294,31 +294,31 @@
     <t>적재</t>
   </si>
   <si>
-    <t>PSIS 문자열 파서 구현</t>
+    <t>엑셀 → JSON 변환 구현 (xlsx_to_json)</t>
   </si>
   <si>
     <t>BE-32</t>
   </si>
   <si>
-    <t>PSIS 농약 데이터 적재 구현</t>
+    <t>엑셀 JSON 약 데이터 적재 구현 (등록·계열)</t>
   </si>
   <si>
     <t>BE-33</t>
   </si>
   <si>
-    <t>NCPMS 병해충 도감 적재 구현</t>
+    <t>엑셀 JSON 병해충 도감·발생시기 적재 구현</t>
   </si>
   <si>
     <t>BE-34</t>
   </si>
   <si>
-    <t>매개충 데이터 작성·적재</t>
+    <t>매개충 데이터 적재 (엑셀 7번)</t>
   </si>
   <si>
     <t>BE-35</t>
   </si>
   <si>
-    <t>작용기작 국제코드 매핑 (별표 8)</t>
+    <t>작용기작 코드 적재 (엑셀 5_약계열)</t>
   </si>
   <si>
     <t>BE-36</t>

</xml_diff>

<commit_message>
Rename docs to Korean titles and update role assignments
Rename the design docs, drop the outline and flow spec, and move zone
detail/update to Hyebin while weather stays with Junhyeok. Align the
architecture doc and the BE backlog (BE-23, BE-28, BE-29) with it.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/dev/farmguardian_backlog_BE.xlsx
+++ b/docs/dev/farmguardian_backlog_BE.xlsx
@@ -270,7 +270,7 @@
     <t>BE-28</t>
   </si>
   <si>
-    <t>구역 서비스 함수 제공 (팀원 연동용)</t>
+    <t>구역 서비스 함수 구현 (구역 생성·요약·위치)</t>
   </si>
   <si>
     <t>BE-29</t>
@@ -1508,7 +1508,7 @@
         <v>10</v>
       </c>
       <c r="E24" s="2" t="s">
-        <v>27</v>
+        <v>11</v>
       </c>
       <c r="F24" s="2" t="s">
         <v>34</v>
@@ -1623,7 +1623,7 @@
         <v>10</v>
       </c>
       <c r="E29" s="2" t="s">
-        <v>11</v>
+        <v>27</v>
       </c>
       <c r="F29" s="2" t="s">
         <v>62</v>
@@ -1646,7 +1646,7 @@
         <v>10</v>
       </c>
       <c r="E30" s="2" t="s">
-        <v>11</v>
+        <v>27</v>
       </c>
       <c r="F30" s="2" t="s">
         <v>62</v>

</xml_diff>

<commit_message>
Update the BE backlog
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/dev/farmguardian_backlog_BE.xlsx
+++ b/docs/dev/farmguardian_backlog_BE.xlsx
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="360" uniqueCount="151">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="354" uniqueCount="151">
   <si>
     <t>ID</t>
   </si>
@@ -294,31 +294,31 @@
     <t>적재</t>
   </si>
   <si>
-    <t>엑셀 → JSON 변환 구현 (xlsx_to_json)</t>
+    <t>(폐기) 엑셀 → JSON 변환 구현 (xlsx_to_json)</t>
   </si>
   <si>
     <t>BE-32</t>
   </si>
   <si>
-    <t>엑셀 JSON 약 데이터 적재 구현 (등록·계열)</t>
+    <t>(폐기) 엑셀 JSON 약 데이터 적재 구현 (등록·계열)</t>
   </si>
   <si>
     <t>BE-33</t>
   </si>
   <si>
-    <t>엑셀 JSON 병해충 도감·발생시기 적재 구현</t>
+    <t>(폐기) 엑셀 JSON 병해충 도감·발생시기 적재 구현</t>
   </si>
   <si>
     <t>BE-34</t>
   </si>
   <si>
-    <t>매개충 데이터 적재 (엑셀 7번)</t>
+    <t>(폐기) 매개충 데이터 적재 (엑셀 7번)</t>
   </si>
   <si>
     <t>BE-35</t>
   </si>
   <si>
-    <t>작용기작 코드 적재 (엑셀 5_약계열)</t>
+    <t>(폐기) 작용기작 코드 적재 (엑셀 5_약계열)</t>
   </si>
   <si>
     <t>BE-36</t>
@@ -953,7 +953,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G55"/>
+  <dimension ref="A1:G54"/>
   <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="8.75" customWidth="1"/>
@@ -1013,13 +1013,13 @@
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="B3" s="2" t="s">
         <v>8</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="D3" s="2" t="s">
         <v>10</v>
@@ -1031,18 +1031,18 @@
         <v>12</v>
       </c>
       <c r="G3" s="2" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="B4" s="2" t="s">
         <v>8</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="D4" s="2" t="s">
         <v>10</v>
@@ -1059,19 +1059,19 @@
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="B5" s="2" t="s">
         <v>8</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="D5" s="2" t="s">
         <v>10</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>11</v>
+        <v>21</v>
       </c>
       <c r="F5" s="2" t="s">
         <v>12</v>
@@ -1082,13 +1082,13 @@
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="B6" s="2" t="s">
         <v>8</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="D6" s="2" t="s">
         <v>10</v>
@@ -1100,24 +1100,24 @@
         <v>12</v>
       </c>
       <c r="G6" s="2" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>8</v>
+        <v>25</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="D7" s="2" t="s">
         <v>10</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="F7" s="2" t="s">
         <v>12</v>
@@ -1128,13 +1128,13 @@
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A8" s="2" t="s">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="B8" s="2" t="s">
         <v>25</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="D8" s="2" t="s">
         <v>10</v>
@@ -1151,13 +1151,13 @@
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A9" s="2" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="B9" s="2" t="s">
         <v>25</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="D9" s="2" t="s">
         <v>10</v>
@@ -1174,22 +1174,22 @@
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A10" s="2" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="B10" s="2" t="s">
         <v>25</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="D10" s="2" t="s">
         <v>10</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>27</v>
+        <v>11</v>
       </c>
       <c r="F10" s="2" t="s">
-        <v>12</v>
+        <v>34</v>
       </c>
       <c r="G10" s="2" t="b">
         <v>0</v>
@@ -1197,22 +1197,22 @@
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A11" s="2" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="B11" s="2" t="s">
         <v>25</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>10</v>
+        <v>37</v>
       </c>
       <c r="E11" s="2" t="s">
         <v>11</v>
       </c>
       <c r="F11" s="2" t="s">
-        <v>34</v>
+        <v>38</v>
       </c>
       <c r="G11" s="2" t="b">
         <v>0</v>
@@ -1220,42 +1220,42 @@
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A12" s="2" t="s">
-        <v>35</v>
+        <v>39</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>25</v>
+        <v>40</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>36</v>
+        <v>41</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>37</v>
+        <v>10</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>11</v>
+        <v>21</v>
       </c>
       <c r="F12" s="2" t="s">
-        <v>38</v>
+        <v>12</v>
       </c>
       <c r="G12" s="2" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A13" s="2" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="B13" s="2" t="s">
         <v>40</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="D13" s="2" t="s">
         <v>10</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>21</v>
+        <v>11</v>
       </c>
       <c r="F13" s="2" t="s">
         <v>12</v>
@@ -1266,19 +1266,19 @@
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A14" s="2" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="B14" s="2" t="s">
         <v>40</v>
       </c>
       <c r="C14" s="3" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="D14" s="2" t="s">
         <v>10</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>11</v>
+        <v>27</v>
       </c>
       <c r="F14" s="2" t="s">
         <v>12</v>
@@ -1289,36 +1289,36 @@
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A15" s="2" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="B15" s="2" t="s">
         <v>40</v>
       </c>
       <c r="C15" s="3" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="D15" s="2" t="s">
         <v>10</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>27</v>
+        <v>11</v>
       </c>
       <c r="F15" s="2" t="s">
         <v>12</v>
       </c>
       <c r="G15" s="2" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A16" s="2" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="B16" s="2" t="s">
         <v>40</v>
       </c>
       <c r="C16" s="3" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="D16" s="2" t="s">
         <v>10</v>
@@ -1330,18 +1330,18 @@
         <v>12</v>
       </c>
       <c r="G16" s="2" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A17" s="2" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>40</v>
+        <v>51</v>
       </c>
       <c r="C17" s="3" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="D17" s="2" t="s">
         <v>10</v>
@@ -1350,21 +1350,21 @@
         <v>11</v>
       </c>
       <c r="F17" s="2" t="s">
-        <v>12</v>
+        <v>34</v>
       </c>
       <c r="G17" s="2" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A18" s="2" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="B18" s="2" t="s">
         <v>51</v>
       </c>
       <c r="C18" s="3" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="D18" s="2" t="s">
         <v>10</v>
@@ -1376,18 +1376,18 @@
         <v>34</v>
       </c>
       <c r="G18" s="2" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A19" s="2" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="B19" s="2" t="s">
         <v>51</v>
       </c>
       <c r="C19" s="3" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="D19" s="2" t="s">
         <v>10</v>
@@ -1399,27 +1399,27 @@
         <v>34</v>
       </c>
       <c r="G19" s="2" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A20" s="2" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>51</v>
+        <v>58</v>
       </c>
       <c r="C20" s="3" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="D20" s="2" t="s">
         <v>10</v>
       </c>
       <c r="E20" s="2" t="s">
-        <v>11</v>
+        <v>27</v>
       </c>
       <c r="F20" s="2" t="s">
-        <v>34</v>
+        <v>12</v>
       </c>
       <c r="G20" s="2" t="b">
         <v>0</v>
@@ -1427,13 +1427,13 @@
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A21" s="2" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="B21" s="2" t="s">
         <v>58</v>
       </c>
       <c r="C21" s="3" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="D21" s="2" t="s">
         <v>10</v>
@@ -1442,21 +1442,21 @@
         <v>27</v>
       </c>
       <c r="F21" s="2" t="s">
-        <v>12</v>
+        <v>62</v>
       </c>
       <c r="G21" s="2" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A22" s="2" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="B22" s="2" t="s">
         <v>58</v>
       </c>
       <c r="C22" s="3" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="D22" s="2" t="s">
         <v>10</v>
@@ -1473,22 +1473,22 @@
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A23" s="2" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="B23" s="2" t="s">
         <v>58</v>
       </c>
       <c r="C23" s="3" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="D23" s="2" t="s">
         <v>10</v>
       </c>
       <c r="E23" s="2" t="s">
-        <v>27</v>
+        <v>11</v>
       </c>
       <c r="F23" s="2" t="s">
-        <v>62</v>
+        <v>34</v>
       </c>
       <c r="G23" s="2" t="b">
         <v>0</v>
@@ -1496,22 +1496,22 @@
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A24" s="2" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>58</v>
+        <v>68</v>
       </c>
       <c r="C24" s="3" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="D24" s="2" t="s">
         <v>10</v>
       </c>
       <c r="E24" s="2" t="s">
-        <v>11</v>
+        <v>27</v>
       </c>
       <c r="F24" s="2" t="s">
-        <v>34</v>
+        <v>62</v>
       </c>
       <c r="G24" s="2" t="b">
         <v>0</v>
@@ -1519,13 +1519,13 @@
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A25" s="2" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="B25" s="2" t="s">
         <v>68</v>
       </c>
       <c r="C25" s="3" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="D25" s="2" t="s">
         <v>10</v>
@@ -1542,13 +1542,13 @@
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A26" s="2" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="B26" s="2" t="s">
         <v>68</v>
       </c>
       <c r="C26" s="3" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="D26" s="2" t="s">
         <v>10</v>
@@ -1565,13 +1565,13 @@
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A27" s="2" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="B27" s="2" t="s">
         <v>68</v>
       </c>
       <c r="C27" s="3" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="D27" s="2" t="s">
         <v>10</v>
@@ -1588,13 +1588,13 @@
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A28" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="B28" s="2" t="s">
         <v>68</v>
       </c>
       <c r="C28" s="3" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="D28" s="2" t="s">
         <v>10</v>
@@ -1611,13 +1611,13 @@
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A29" s="2" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="B29" s="2" t="s">
         <v>68</v>
       </c>
       <c r="C29" s="3" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="D29" s="2" t="s">
         <v>10</v>
@@ -1634,22 +1634,22 @@
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A30" s="2" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="B30" s="2" t="s">
         <v>68</v>
       </c>
       <c r="C30" s="3" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="D30" s="2" t="s">
-        <v>10</v>
+        <v>82</v>
       </c>
       <c r="E30" s="2" t="s">
         <v>27</v>
       </c>
       <c r="F30" s="2" t="s">
-        <v>62</v>
+        <v>38</v>
       </c>
       <c r="G30" s="2" t="b">
         <v>0</v>
@@ -1657,22 +1657,22 @@
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A31" s="2" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>68</v>
+        <v>84</v>
       </c>
       <c r="C31" s="3" t="s">
-        <v>81</v>
+        <v>85</v>
       </c>
       <c r="D31" s="2" t="s">
-        <v>82</v>
+        <v>10</v>
       </c>
       <c r="E31" s="2" t="s">
-        <v>27</v>
+        <v>11</v>
       </c>
       <c r="F31" s="2" t="s">
-        <v>38</v>
+        <v>12</v>
       </c>
       <c r="G31" s="2" t="b">
         <v>0</v>
@@ -1680,13 +1680,13 @@
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A32" s="2" t="s">
-        <v>83</v>
+        <v>86</v>
       </c>
       <c r="B32" s="2" t="s">
         <v>84</v>
       </c>
       <c r="C32" s="3" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="D32" s="2" t="s">
         <v>10</v>
@@ -1695,7 +1695,7 @@
         <v>11</v>
       </c>
       <c r="F32" s="2" t="s">
-        <v>12</v>
+        <v>62</v>
       </c>
       <c r="G32" s="2" t="b">
         <v>0</v>
@@ -1703,13 +1703,13 @@
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A33" s="2" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="B33" s="2" t="s">
         <v>84</v>
       </c>
       <c r="C33" s="3" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="D33" s="2" t="s">
         <v>10</v>
@@ -1718,7 +1718,7 @@
         <v>11</v>
       </c>
       <c r="F33" s="2" t="s">
-        <v>62</v>
+        <v>34</v>
       </c>
       <c r="G33" s="2" t="b">
         <v>0</v>
@@ -1726,13 +1726,13 @@
     </row>
     <row r="34" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A34" s="2" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="B34" s="2" t="s">
         <v>84</v>
       </c>
       <c r="C34" s="3" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="D34" s="2" t="s">
         <v>10</v>
@@ -1749,13 +1749,13 @@
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A35" s="2" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="B35" s="2" t="s">
         <v>84</v>
       </c>
       <c r="C35" s="3" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="D35" s="2" t="s">
         <v>10</v>
@@ -1772,13 +1772,13 @@
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A36" s="2" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="B36" s="2" t="s">
-        <v>84</v>
+        <v>95</v>
       </c>
       <c r="C36" s="3" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="D36" s="2" t="s">
         <v>10</v>
@@ -1790,18 +1790,18 @@
         <v>34</v>
       </c>
       <c r="G36" s="2" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A37" s="2" t="s">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="B37" s="2" t="s">
         <v>95</v>
       </c>
       <c r="C37" s="3" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="D37" s="2" t="s">
         <v>10</v>
@@ -1810,21 +1810,21 @@
         <v>11</v>
       </c>
       <c r="F37" s="2" t="s">
-        <v>34</v>
+        <v>62</v>
       </c>
       <c r="G37" s="2" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A38" s="2" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="B38" s="2" t="s">
-        <v>95</v>
+        <v>100</v>
       </c>
       <c r="C38" s="3" t="s">
-        <v>98</v>
+        <v>101</v>
       </c>
       <c r="D38" s="2" t="s">
         <v>10</v>
@@ -1833,21 +1833,21 @@
         <v>11</v>
       </c>
       <c r="F38" s="2" t="s">
-        <v>62</v>
+        <v>12</v>
       </c>
       <c r="G38" s="2" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="39" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A39" s="2" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
       <c r="B39" s="2" t="s">
         <v>100</v>
       </c>
       <c r="C39" s="3" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="D39" s="2" t="s">
         <v>10</v>
@@ -1859,18 +1859,18 @@
         <v>12</v>
       </c>
       <c r="G39" s="2" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="40" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A40" s="2" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="B40" s="2" t="s">
         <v>100</v>
       </c>
       <c r="C40" s="3" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="D40" s="2" t="s">
         <v>10</v>
@@ -1879,21 +1879,21 @@
         <v>11</v>
       </c>
       <c r="F40" s="2" t="s">
-        <v>12</v>
+        <v>62</v>
       </c>
       <c r="G40" s="2" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="41" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A41" s="2" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="B41" s="2" t="s">
         <v>100</v>
       </c>
       <c r="C41" s="3" t="s">
-        <v>105</v>
+        <v>150</v>
       </c>
       <c r="D41" s="2" t="s">
         <v>10</v>
@@ -1905,18 +1905,18 @@
         <v>62</v>
       </c>
       <c r="G41" s="2" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A42" s="2" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="B42" s="2" t="s">
         <v>100</v>
       </c>
       <c r="C42" s="3" t="s">
-        <v>150</v>
+        <v>108</v>
       </c>
       <c r="D42" s="2" t="s">
         <v>10</v>
@@ -1928,18 +1928,18 @@
         <v>62</v>
       </c>
       <c r="G42" s="2" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A43" s="2" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="B43" s="2" t="s">
         <v>100</v>
       </c>
       <c r="C43" s="3" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="D43" s="2" t="s">
         <v>10</v>
@@ -1951,18 +1951,18 @@
         <v>62</v>
       </c>
       <c r="G43" s="2" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="44" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A44" s="2" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="B44" s="2" t="s">
         <v>100</v>
       </c>
       <c r="C44" s="3" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="D44" s="2" t="s">
         <v>10</v>
@@ -1974,18 +1974,18 @@
         <v>62</v>
       </c>
       <c r="G44" s="2" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="45" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A45" s="2" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="B45" s="2" t="s">
         <v>100</v>
       </c>
       <c r="C45" s="3" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="D45" s="2" t="s">
         <v>10</v>
@@ -1997,18 +1997,18 @@
         <v>62</v>
       </c>
       <c r="G45" s="2" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="46" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A46" s="2" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="B46" s="2" t="s">
-        <v>100</v>
+        <v>116</v>
       </c>
       <c r="C46" s="3" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="D46" s="2" t="s">
         <v>10</v>
@@ -2020,18 +2020,18 @@
         <v>62</v>
       </c>
       <c r="G46" s="2" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="47" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A47" s="2" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="B47" s="2" t="s">
         <v>116</v>
       </c>
       <c r="C47" s="3" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="D47" s="2" t="s">
         <v>10</v>
@@ -2043,27 +2043,27 @@
         <v>62</v>
       </c>
       <c r="G47" s="2" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="48" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A48" s="2" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="B48" s="2" t="s">
-        <v>116</v>
+        <v>121</v>
       </c>
       <c r="C48" s="3" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="D48" s="2" t="s">
         <v>10</v>
       </c>
       <c r="E48" s="2" t="s">
-        <v>11</v>
+        <v>27</v>
       </c>
       <c r="F48" s="2" t="s">
-        <v>62</v>
+        <v>34</v>
       </c>
       <c r="G48" s="2" t="b">
         <v>0</v>
@@ -2071,36 +2071,36 @@
     </row>
     <row r="49" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A49" s="2" t="s">
-        <v>120</v>
+        <v>123</v>
       </c>
       <c r="B49" s="2" t="s">
         <v>121</v>
       </c>
       <c r="C49" s="3" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="D49" s="2" t="s">
         <v>10</v>
       </c>
       <c r="E49" s="2" t="s">
-        <v>27</v>
+        <v>11</v>
       </c>
       <c r="F49" s="2" t="s">
         <v>34</v>
       </c>
       <c r="G49" s="2" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="50" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A50" s="2" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="B50" s="2" t="s">
         <v>121</v>
       </c>
       <c r="C50" s="3" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="D50" s="2" t="s">
         <v>10</v>
@@ -2117,19 +2117,19 @@
     </row>
     <row r="51" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A51" s="2" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="B51" s="2" t="s">
         <v>121</v>
       </c>
       <c r="C51" s="3" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="D51" s="2" t="s">
         <v>10</v>
       </c>
       <c r="E51" s="2" t="s">
-        <v>11</v>
+        <v>129</v>
       </c>
       <c r="F51" s="2" t="s">
         <v>34</v>
@@ -2140,22 +2140,22 @@
     </row>
     <row r="52" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A52" s="2" t="s">
-        <v>127</v>
+        <v>130</v>
       </c>
       <c r="B52" s="2" t="s">
-        <v>121</v>
+        <v>131</v>
       </c>
       <c r="C52" s="3" t="s">
-        <v>128</v>
+        <v>132</v>
       </c>
       <c r="D52" s="2" t="s">
         <v>10</v>
       </c>
       <c r="E52" s="2" t="s">
-        <v>129</v>
+        <v>11</v>
       </c>
       <c r="F52" s="2" t="s">
-        <v>34</v>
+        <v>12</v>
       </c>
       <c r="G52" s="2" t="b">
         <v>0</v>
@@ -2163,13 +2163,13 @@
     </row>
     <row r="53" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A53" s="2" t="s">
-        <v>130</v>
+        <v>133</v>
       </c>
       <c r="B53" s="2" t="s">
         <v>131</v>
       </c>
       <c r="C53" s="3" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="D53" s="2" t="s">
         <v>10</v>
@@ -2186,52 +2186,29 @@
     </row>
     <row r="54" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A54" s="2" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="B54" s="2" t="s">
         <v>131</v>
       </c>
       <c r="C54" s="3" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="D54" s="2" t="s">
         <v>10</v>
       </c>
       <c r="E54" s="2" t="s">
-        <v>11</v>
+        <v>27</v>
       </c>
       <c r="F54" s="2" t="s">
-        <v>12</v>
+        <v>62</v>
       </c>
       <c r="G54" s="2" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="55" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A55" s="2" t="s">
-        <v>135</v>
-      </c>
-      <c r="B55" s="2" t="s">
-        <v>131</v>
-      </c>
-      <c r="C55" s="3" t="s">
-        <v>136</v>
-      </c>
-      <c r="D55" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="E55" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="F55" s="2" t="s">
-        <v>62</v>
-      </c>
-      <c r="G55" s="2" t="b">
-        <v>0</v>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:G55" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
+  <autoFilter ref="A1:G54" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
   <phoneticPr fontId="6" type="noConversion"/>
   <conditionalFormatting sqref="A2:G300">
     <cfRule type="expression" dxfId="0" priority="1">
@@ -2292,15 +2269,15 @@
       </c>
       <c r="B5" s="2">
         <f>COUNTIF(백로그!$F$2:$F$300,A5)</f>
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C5" s="2">
         <f>COUNTIFS(백로그!$F$2:$F$300,A5,백로그!$G$2:$G$300,TRUE)</f>
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="D5" s="7">
         <f>IFERROR(C5/B5,0)</f>
-        <v>0.1</v>
+        <v>0.47368421052631576</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.3">
@@ -2313,11 +2290,11 @@
       </c>
       <c r="C6" s="2">
         <f>COUNTIFS(백로그!$F$2:$F$300,A6,백로그!$G$2:$G$300,TRUE)</f>
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="D6" s="7">
         <f>IFERROR(C6/B6,0)</f>
-        <v>0</v>
+        <v>0.5263157894736842</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.3">
@@ -2330,11 +2307,11 @@
       </c>
       <c r="C7" s="2">
         <f>COUNTIFS(백로그!$F$2:$F$300,A7,백로그!$G$2:$G$300,TRUE)</f>
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D7" s="7">
         <f>IFERROR(C7/B7,0)</f>
-        <v>0</v>
+        <v>0.38461538461538464</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.3">
@@ -2351,7 +2328,7 @@
       </c>
       <c r="D8" s="7">
         <f>IFERROR(C8/B8,0)</f>
-        <v>0</v>
+        <v>0.0</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.3">
@@ -2360,15 +2337,15 @@
       </c>
       <c r="B9" s="8">
         <f>COUNTA(백로그!$A$2:$A$300)</f>
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C9" s="8">
         <f>COUNTIF(백로그!$G$2:$G$300,TRUE)</f>
-        <v>2</v>
+        <v>24</v>
       </c>
       <c r="D9" s="9">
         <f>IFERROR(C9/B9,0)</f>
-        <v>3.7037037037037035E-2</v>
+        <v>0.4528301886792453</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.3">

</xml_diff>